<commit_message>
feat: add dynamic Streamlit app, streamline docs and power bi files for neat presentation
</commit_message>
<xml_diff>
--- a/excel/swiggy_business_performance_review.xlsx
+++ b/excel/swiggy_business_performance_review.xlsx
@@ -36,7 +36,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -48,7 +48,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="001F2937"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -564,7 +564,7 @@
   <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Annual Business Review &amp; Marketplace Metrics (FY 2024)</t>
+          <t>Marketplace Analytics &amp; Financial Review — Prepared by Disha Gomes</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Revenue &amp; Cost Drivers (Unit Economics)</t>
+          <t>Revenue &amp; Cost Drivers (Prepared by Disha Gomes)</t>
         </is>
       </c>
     </row>

</xml_diff>